<commit_message>
Release South installation type field 0.9.57
</commit_message>
<xml_diff>
--- a/MN/Giao_phieu_MN.xlsx
+++ b/MN/Giao_phieu_MN.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tranmanhcuong/Projects/ATS_OneBss/MN/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44EA7209-4B2D-9B45-A715-6430347AF1BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5852989-D79C-FB4D-A39A-908D665E85D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51200" yWindow="10300" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="51200" yWindow="10300" windowWidth="30240" windowHeight="18980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Quy tắc giao phiếu_MN" sheetId="3" r:id="rId1"/>
     <sheet name="Group DV" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Group DV'!$A$1:$F$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Group DV'!$A$1:$F$62</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Quy tắc giao phiếu_MN'!$A$2:$M$31</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="93">
   <si>
     <t>STT</t>
   </si>
@@ -314,6 +314,9 @@
   </si>
   <si>
     <t>Phạm Thị Thiên Linh</t>
+  </si>
+  <si>
+    <t>Leasedline 100GE</t>
   </si>
 </sst>
 </file>
@@ -1698,7 +1701,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DE81EBB-08AC-CB41-ACC3-3E8E86C36875}">
-  <dimension ref="A1:F61"/>
+  <dimension ref="A1:F62"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
@@ -2231,18 +2234,18 @@
       <c r="A29" s="7">
         <v>28</v>
       </c>
-      <c r="B29" s="5">
-        <v>1800</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D29" s="8">
-        <v>17</v>
-      </c>
-      <c r="E29" s="8"/>
+      <c r="B29" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D29" s="7">
+        <v>42</v>
+      </c>
+      <c r="E29" s="7"/>
       <c r="F29" s="5" t="s">
-        <v>17</v>
+        <v>40</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -2250,7 +2253,7 @@
         <v>29</v>
       </c>
       <c r="B30" s="5">
-        <v>1900</v>
+        <v>1800</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>17</v>
@@ -2267,18 +2270,18 @@
       <c r="A31" s="7">
         <v>30</v>
       </c>
-      <c r="B31" s="5" t="s">
-        <v>32</v>
+      <c r="B31" s="5">
+        <v>1900</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="D31" s="8">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="E31" s="8"/>
       <c r="F31" s="5" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -2286,10 +2289,10 @@
         <v>31</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D32" s="8">
         <v>27</v>
@@ -2304,7 +2307,7 @@
         <v>32</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C33" s="5" t="s">
         <v>34</v>
@@ -2317,24 +2320,22 @@
         <v>34</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="108" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A34" s="7">
         <v>33</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="D34" s="8">
-        <v>14</v>
-      </c>
-      <c r="E34" s="9" t="s">
-        <v>73</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="E34" s="8"/>
       <c r="F34" s="5" t="s">
-        <v>76</v>
+        <v>34</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="108" x14ac:dyDescent="0.2">
@@ -2342,10 +2343,10 @@
         <v>34</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D35" s="8">
         <v>14</v>
@@ -2357,24 +2358,24 @@
         <v>76</v>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="18" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6" ht="108" x14ac:dyDescent="0.2">
       <c r="A36" s="7">
         <v>35</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D36" s="8">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="E36" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="18" x14ac:dyDescent="0.2">
@@ -2382,10 +2383,10 @@
         <v>36</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D37" s="8">
         <v>29</v>
@@ -2397,24 +2398,24 @@
         <v>77</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="36" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A38" s="7">
         <v>37</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D38" s="8">
         <v>29</v>
       </c>
       <c r="E38" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="39" spans="1:6" ht="36" x14ac:dyDescent="0.2">
@@ -2422,10 +2423,10 @@
         <v>38</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D39" s="8">
         <v>29</v>
@@ -2442,19 +2443,19 @@
         <v>39</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="D40" s="8">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="E40" s="9" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="36" x14ac:dyDescent="0.2">
@@ -2462,10 +2463,10 @@
         <v>40</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D41" s="8">
         <v>14</v>
@@ -2477,22 +2478,24 @@
         <v>79</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6" ht="36" x14ac:dyDescent="0.2">
       <c r="A42" s="7">
         <v>41</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>9</v>
+        <v>44</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="D42" s="8">
-        <v>10</v>
-      </c>
-      <c r="E42" s="8"/>
+        <v>14</v>
+      </c>
+      <c r="E42" s="9" t="s">
+        <v>74</v>
+      </c>
       <c r="F42" s="5" t="s">
-        <v>10</v>
+        <v>79</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -2500,7 +2503,7 @@
         <v>42</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C43" s="5" t="s">
         <v>10</v>
@@ -2518,17 +2521,17 @@
         <v>43</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>48</v>
+        <v>11</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>48</v>
+        <v>10</v>
       </c>
       <c r="D44" s="8">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="E44" s="8"/>
       <c r="F44" s="5" t="s">
-        <v>48</v>
+        <v>10</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -2536,7 +2539,7 @@
         <v>44</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="C45" s="5" t="s">
         <v>48</v>
@@ -2554,17 +2557,17 @@
         <v>45</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>5</v>
+        <v>66</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>5</v>
+        <v>48</v>
       </c>
       <c r="D46" s="8">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="E46" s="8"/>
       <c r="F46" s="5" t="s">
-        <v>5</v>
+        <v>48</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -2572,17 +2575,17 @@
         <v>46</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="D47" s="8">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="E47" s="8"/>
       <c r="F47" s="5" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="48" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -2590,17 +2593,17 @@
         <v>47</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D48" s="8">
         <v>17</v>
       </c>
       <c r="E48" s="8"/>
       <c r="F48" s="5" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="49" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -2608,19 +2611,17 @@
         <v>48</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D49" s="8">
-        <v>20</v>
-      </c>
-      <c r="E49" s="8" t="s">
-        <v>80</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="E49" s="8"/>
       <c r="F49" s="5" t="s">
-        <v>82</v>
+        <v>16</v>
       </c>
     </row>
     <row r="50" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -2637,10 +2638,10 @@
         <v>20</v>
       </c>
       <c r="E50" s="8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F50" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -2648,17 +2649,19 @@
         <v>50</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D51" s="8">
-        <v>17</v>
-      </c>
-      <c r="E51" s="8"/>
+        <v>20</v>
+      </c>
+      <c r="E51" s="8" t="s">
+        <v>81</v>
+      </c>
       <c r="F51" s="5" t="s">
-        <v>19</v>
+        <v>83</v>
       </c>
     </row>
     <row r="52" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -2666,17 +2669,17 @@
         <v>51</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D52" s="8">
         <v>17</v>
       </c>
       <c r="E52" s="8"/>
       <c r="F52" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="53" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -2684,17 +2687,17 @@
         <v>52</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D53" s="8">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="E53" s="8"/>
       <c r="F53" s="5" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
     </row>
     <row r="54" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -2702,17 +2705,17 @@
         <v>53</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="D54" s="8">
         <v>27</v>
       </c>
       <c r="E54" s="8"/>
       <c r="F54" s="5" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
     </row>
     <row r="55" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -2720,17 +2723,17 @@
         <v>54</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="D55" s="8">
         <v>27</v>
       </c>
       <c r="E55" s="8"/>
       <c r="F55" s="5" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
     </row>
     <row r="56" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -2738,17 +2741,17 @@
         <v>55</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D56" s="8">
         <v>27</v>
       </c>
       <c r="E56" s="8"/>
       <c r="F56" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="57" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -2756,17 +2759,17 @@
         <v>56</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D57" s="8">
         <v>27</v>
       </c>
       <c r="E57" s="8"/>
       <c r="F57" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="58" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -2774,17 +2777,17 @@
         <v>57</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="D58" s="8">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E58" s="8"/>
       <c r="F58" s="5" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
     </row>
     <row r="59" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -2792,33 +2795,35 @@
         <v>58</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D59" s="8">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="E59" s="8"/>
       <c r="F59" s="5" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="60" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A60" s="7">
         <v>59</v>
       </c>
-      <c r="B60" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="C60" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="D60" s="7"/>
-      <c r="E60" s="7"/>
-      <c r="F60" s="7" t="s">
-        <v>60</v>
+      <c r="B60" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C60" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D60" s="8">
+        <v>14</v>
+      </c>
+      <c r="E60" s="8"/>
+      <c r="F60" s="5" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="61" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -2826,19 +2831,35 @@
         <v>60</v>
       </c>
       <c r="B61" s="7" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C61" s="7" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D61" s="7"/>
       <c r="E61" s="7"/>
       <c r="F61" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="A62" s="7">
+        <v>61</v>
+      </c>
+      <c r="B62" s="7" t="s">
         <v>64</v>
       </c>
+      <c r="C62" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="D62" s="7"/>
+      <c r="E62" s="7"/>
+      <c r="F62" s="7" t="s">
+        <v>64</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F61" xr:uid="{4DE81EBB-08AC-CB41-ACC3-3E8E86C36875}"/>
+  <autoFilter ref="A1:F62" xr:uid="{4DE81EBB-08AC-CB41-ACC3-3E8E86C36875}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>